<commit_message>
chore(data-release): publish site data 2026-10-08 00:23:38 UTC
</commit_message>
<xml_diff>
--- a/countries/cn-ah/2000-2004.xlsx
+++ b/countries/cn-ah/2000-2004.xlsx
@@ -765,9 +765,12 @@
       <c r="O2" t="n">
         <v>243</v>
       </c>
+      <c r="R2" t="n">
+        <v>0.3901734104046242</v>
+      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -1150,9 +1153,12 @@
       <c r="O4" t="n">
         <v>2573</v>
       </c>
+      <c r="R4" t="n">
+        <v>4.131342324983944</v>
+      </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -1535,9 +1541,12 @@
       <c r="O6" t="n">
         <v>41</v>
       </c>
+      <c r="R6" t="n">
+        <v>0.06583172768143866</v>
+      </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -1920,9 +1929,12 @@
       <c r="O8" t="n">
         <v>49</v>
       </c>
+      <c r="R8" t="n">
+        <v>0.07867694283879255</v>
+      </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -2305,9 +2317,12 @@
       <c r="O10" t="n">
         <v>441</v>
       </c>
+      <c r="R10" t="n">
+        <v>0.708092485549133</v>
+      </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -2690,9 +2705,12 @@
       <c r="O12" t="n">
         <v>3145</v>
       </c>
+      <c r="R12" t="n">
+        <v>5.049775208734746</v>
+      </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
@@ -3075,9 +3093,12 @@
       <c r="O14" t="n">
         <v>11</v>
       </c>
+      <c r="R14" t="n">
+        <v>0.01766217084136159</v>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
@@ -3460,9 +3481,12 @@
       <c r="O16" t="n">
         <v>13</v>
       </c>
+      <c r="R16" t="n">
+        <v>0.02087347463070006</v>
+      </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
@@ -3845,9 +3869,12 @@
       <c r="O18" t="n">
         <v>581</v>
       </c>
+      <c r="R18" t="n">
+        <v>0.932883750802826</v>
+      </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
@@ -4230,9 +4257,12 @@
       <c r="O20" t="n">
         <v>181</v>
       </c>
+      <c r="R20" t="n">
+        <v>0.2906229929351317</v>
+      </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
@@ -4615,9 +4645,12 @@
       <c r="O22" t="n">
         <v>20</v>
       </c>
+      <c r="R22" t="n">
+        <v>0.03211303789338472</v>
+      </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
@@ -5000,9 +5033,12 @@
       <c r="O24" t="n">
         <v>153</v>
       </c>
+      <c r="R24" t="n">
+        <v>0.2456647398843931</v>
+      </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
@@ -5385,9 +5421,12 @@
       <c r="O26" t="n">
         <v>6</v>
       </c>
+      <c r="R26" t="n">
+        <v>0.009633911368015413</v>
+      </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
@@ -5770,9 +5809,12 @@
       <c r="O28" t="n">
         <v>11</v>
       </c>
+      <c r="R28" t="n">
+        <v>0.01766217084136159</v>
+      </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
@@ -6155,9 +6197,12 @@
       <c r="O30" t="n">
         <v>106</v>
       </c>
+      <c r="R30" t="n">
+        <v>0.170199100834939</v>
+      </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr">
@@ -6540,9 +6585,12 @@
       <c r="O32" t="n">
         <v>18</v>
       </c>
+      <c r="R32" t="n">
+        <v>0.02890173410404624</v>
+      </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
@@ -6925,9 +6973,12 @@
       <c r="O34" t="n">
         <v>1</v>
       </c>
+      <c r="R34" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
@@ -7310,9 +7361,12 @@
       <c r="O36" t="n">
         <v>333</v>
       </c>
+      <c r="R36" t="n">
+        <v>0.5346820809248555</v>
+      </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
@@ -7695,9 +7749,12 @@
       <c r="O38" t="n">
         <v>2773</v>
       </c>
+      <c r="R38" t="n">
+        <v>4.452472703917791</v>
+      </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
@@ -8080,9 +8137,12 @@
       <c r="O40" t="n">
         <v>55</v>
       </c>
+      <c r="R40" t="n">
+        <v>0.08831085420680797</v>
+      </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA40" t="inlineStr">
@@ -8465,9 +8525,12 @@
       <c r="O42" t="n">
         <v>95</v>
       </c>
+      <c r="R42" t="n">
+        <v>0.1525369299935774</v>
+      </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA42" t="inlineStr">
@@ -8850,9 +8913,12 @@
       <c r="O44" t="n">
         <v>515</v>
       </c>
+      <c r="R44" t="n">
+        <v>0.8269107257546564</v>
+      </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA44" t="inlineStr">
@@ -9235,9 +9301,12 @@
       <c r="O46" t="n">
         <v>2936</v>
       </c>
+      <c r="R46" t="n">
+        <v>4.714193962748876</v>
+      </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA46" t="inlineStr">
@@ -9620,9 +9689,12 @@
       <c r="O48" t="n">
         <v>12</v>
       </c>
+      <c r="R48" t="n">
+        <v>0.01926782273603083</v>
+      </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA48" t="inlineStr">
@@ -10005,9 +10077,12 @@
       <c r="O50" t="n">
         <v>6</v>
       </c>
+      <c r="R50" t="n">
+        <v>0.009633911368015413</v>
+      </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA50" t="inlineStr">
@@ -10390,9 +10465,12 @@
       <c r="O52" t="n">
         <v>23</v>
       </c>
+      <c r="R52" t="n">
+        <v>0.03692999357739242</v>
+      </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA52" t="inlineStr">
@@ -10775,9 +10853,12 @@
       <c r="O54" t="n">
         <v>539</v>
       </c>
+      <c r="R54" t="n">
+        <v>0.865446371226718</v>
+      </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA54" t="inlineStr">
@@ -11160,9 +11241,12 @@
       <c r="O56" t="n">
         <v>214</v>
       </c>
+      <c r="R56" t="n">
+        <v>0.3436095054592165</v>
+      </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA56" t="inlineStr">
@@ -11545,9 +11629,12 @@
       <c r="O58" t="n">
         <v>28</v>
       </c>
+      <c r="R58" t="n">
+        <v>0.0449582530507386</v>
+      </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA58" t="inlineStr">
@@ -11930,9 +12017,12 @@
       <c r="O60" t="n">
         <v>134</v>
       </c>
+      <c r="R60" t="n">
+        <v>0.2151573538856776</v>
+      </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA60" t="inlineStr">
@@ -12315,9 +12405,12 @@
       <c r="O62" t="n">
         <v>19</v>
       </c>
+      <c r="R62" t="n">
+        <v>0.03050738599871548</v>
+      </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA62" t="inlineStr">
@@ -12700,9 +12793,12 @@
       <c r="O64" t="n">
         <v>8</v>
       </c>
+      <c r="R64" t="n">
+        <v>0.01284521515735389</v>
+      </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA64" t="inlineStr">
@@ -13085,9 +13181,12 @@
       <c r="O66" t="n">
         <v>112</v>
       </c>
+      <c r="R66" t="n">
+        <v>0.1798330122029544</v>
+      </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA66" t="inlineStr">
@@ -13470,9 +13569,12 @@
       <c r="O68" t="n">
         <v>8</v>
       </c>
+      <c r="R68" t="n">
+        <v>0.01284521515735389</v>
+      </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA68" t="inlineStr">
@@ -13855,9 +13957,12 @@
       <c r="O70" t="n">
         <v>1</v>
       </c>
+      <c r="R70" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA70" t="inlineStr">
@@ -14240,9 +14345,12 @@
       <c r="O72" t="n">
         <v>388</v>
       </c>
+      <c r="R72" t="n">
+        <v>0.6229929351316634</v>
+      </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA72" t="inlineStr">
@@ -14625,9 +14733,12 @@
       <c r="O74" t="n">
         <v>2817</v>
       </c>
+      <c r="R74" t="n">
+        <v>4.523121387283237</v>
+      </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA74" t="inlineStr">
@@ -15010,9 +15121,12 @@
       <c r="O76" t="n">
         <v>64</v>
       </c>
+      <c r="R76" t="n">
+        <v>0.1027617212588311</v>
+      </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA76" t="inlineStr">
@@ -15395,9 +15509,12 @@
       <c r="O78" t="n">
         <v>103</v>
       </c>
+      <c r="R78" t="n">
+        <v>0.1653821451509313</v>
+      </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA78" t="inlineStr">
@@ -15780,9 +15897,12 @@
       <c r="O80" t="n">
         <v>564</v>
       </c>
+      <c r="R80" t="n">
+        <v>0.9055876685934489</v>
+      </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA80" t="inlineStr">
@@ -16165,9 +16285,12 @@
       <c r="O82" t="n">
         <v>3213</v>
       </c>
+      <c r="R82" t="n">
+        <v>5.158959537572255</v>
+      </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA82" t="inlineStr">
@@ -16550,9 +16673,12 @@
       <c r="O84" t="n">
         <v>19</v>
       </c>
+      <c r="R84" t="n">
+        <v>0.03050738599871548</v>
+      </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA84" t="inlineStr">
@@ -16935,9 +17061,12 @@
       <c r="O86" t="n">
         <v>9</v>
       </c>
+      <c r="R86" t="n">
+        <v>0.01445086705202312</v>
+      </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA86" t="inlineStr">
@@ -17320,9 +17449,12 @@
       <c r="O88" t="n">
         <v>31</v>
       </c>
+      <c r="R88" t="n">
+        <v>0.04977520873474631</v>
+      </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA88" t="inlineStr">
@@ -17705,9 +17837,12 @@
       <c r="O90" t="n">
         <v>632</v>
       </c>
+      <c r="R90" t="n">
+        <v>1.014771997430957</v>
+      </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA90" t="inlineStr">
@@ -18090,9 +18225,12 @@
       <c r="O92" t="n">
         <v>236</v>
       </c>
+      <c r="R92" t="n">
+        <v>0.3789338471419396</v>
+      </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA92" t="inlineStr">
@@ -18475,9 +18613,12 @@
       <c r="O94" t="n">
         <v>52</v>
       </c>
+      <c r="R94" t="n">
+        <v>0.08349389852280026</v>
+      </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA94" t="inlineStr">
@@ -18860,9 +19001,12 @@
       <c r="O96" t="n">
         <v>427</v>
       </c>
+      <c r="R96" t="n">
+        <v>0.6856133590237636</v>
+      </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA96" t="inlineStr">
@@ -19245,9 +19389,12 @@
       <c r="O98" t="n">
         <v>47</v>
       </c>
+      <c r="R98" t="n">
+        <v>0.07546563904945408</v>
+      </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA98" t="inlineStr">
@@ -19630,9 +19777,12 @@
       <c r="O100" t="n">
         <v>28</v>
       </c>
+      <c r="R100" t="n">
+        <v>0.0449582530507386</v>
+      </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA100" t="inlineStr">
@@ -20015,9 +20165,12 @@
       <c r="O102" t="n">
         <v>208</v>
       </c>
+      <c r="R102" t="n">
+        <v>0.333975594091201</v>
+      </c>
       <c r="S102" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA102" t="inlineStr">
@@ -20400,9 +20553,12 @@
       <c r="O104" t="n">
         <v>18</v>
       </c>
+      <c r="R104" t="n">
+        <v>0.02890173410404624</v>
+      </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA104" t="inlineStr">
@@ -20785,9 +20941,12 @@
       <c r="O106" t="n">
         <v>1</v>
       </c>
+      <c r="R106" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S106" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA106" t="inlineStr">
@@ -21170,9 +21329,12 @@
       <c r="O108" t="n">
         <v>358</v>
       </c>
+      <c r="R108" t="n">
+        <v>0.5748233782915864</v>
+      </c>
       <c r="S108" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA108" t="inlineStr">
@@ -21555,9 +21717,12 @@
       <c r="O110" t="n">
         <v>3121</v>
       </c>
+      <c r="R110" t="n">
+        <v>5.011239563262685</v>
+      </c>
       <c r="S110" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA110" t="inlineStr">
@@ -21940,9 +22105,12 @@
       <c r="O112" t="n">
         <v>68</v>
       </c>
+      <c r="R112" t="n">
+        <v>0.109184328837508</v>
+      </c>
       <c r="S112" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA112" t="inlineStr">
@@ -22325,9 +22493,12 @@
       <c r="O114" t="n">
         <v>99</v>
       </c>
+      <c r="R114" t="n">
+        <v>0.1589595375722543</v>
+      </c>
       <c r="S114" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA114" t="inlineStr">
@@ -22710,9 +22881,12 @@
       <c r="O116" t="n">
         <v>860</v>
       </c>
+      <c r="R116" t="n">
+        <v>1.380860629415543</v>
+      </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA116" t="inlineStr">
@@ -23095,9 +23269,12 @@
       <c r="O118" t="n">
         <v>3365</v>
       </c>
+      <c r="R118" t="n">
+        <v>5.403018625561979</v>
+      </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA118" t="inlineStr">
@@ -23480,9 +23657,12 @@
       <c r="O120" t="n">
         <v>23</v>
       </c>
+      <c r="R120" t="n">
+        <v>0.03692999357739242</v>
+      </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA120" t="inlineStr">
@@ -23865,9 +24045,12 @@
       <c r="O122" t="n">
         <v>24</v>
       </c>
+      <c r="R122" t="n">
+        <v>0.03853564547206165</v>
+      </c>
       <c r="S122" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA122" t="inlineStr">
@@ -24250,9 +24433,12 @@
       <c r="O124" t="n">
         <v>37</v>
       </c>
+      <c r="R124" t="n">
+        <v>0.05940912010276172</v>
+      </c>
       <c r="S124" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA124" t="inlineStr">
@@ -24635,9 +24821,12 @@
       <c r="O126" t="n">
         <v>772</v>
       </c>
+      <c r="R126" t="n">
+        <v>1.23956326268465</v>
+      </c>
       <c r="S126" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA126" t="inlineStr">
@@ -25020,9 +25209,12 @@
       <c r="O128" t="n">
         <v>293</v>
       </c>
+      <c r="R128" t="n">
+        <v>0.4704560051380861</v>
+      </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA128" t="inlineStr">
@@ -25405,9 +25597,12 @@
       <c r="O130" t="n">
         <v>159</v>
       </c>
+      <c r="R130" t="n">
+        <v>0.2552986512524085</v>
+      </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA130" t="inlineStr">
@@ -25790,9 +25985,12 @@
       <c r="O132" t="n">
         <v>1015</v>
       </c>
+      <c r="R132" t="n">
+        <v>1.629736673089274</v>
+      </c>
       <c r="S132" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA132" t="inlineStr">
@@ -26175,9 +26373,12 @@
       <c r="O134" t="n">
         <v>103</v>
       </c>
+      <c r="R134" t="n">
+        <v>0.1653821451509313</v>
+      </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA134" t="inlineStr">
@@ -26560,9 +26761,12 @@
       <c r="O136" t="n">
         <v>22</v>
       </c>
+      <c r="R136" t="n">
+        <v>0.03532434168272319</v>
+      </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA136" t="inlineStr">
@@ -26945,9 +27149,12 @@
       <c r="O138" t="n">
         <v>557</v>
       </c>
+      <c r="R138" t="n">
+        <v>0.8943481053307643</v>
+      </c>
       <c r="S138" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA138" t="inlineStr">
@@ -27330,9 +27537,12 @@
       <c r="O140" t="n">
         <v>26</v>
       </c>
+      <c r="R140" t="n">
+        <v>0.04174694926140013</v>
+      </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA140" t="inlineStr">
@@ -27715,9 +27925,12 @@
       <c r="O142" t="n">
         <v>419</v>
       </c>
+      <c r="R142" t="n">
+        <v>0.6727681438664097</v>
+      </c>
       <c r="S142" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA142" t="inlineStr">
@@ -28100,9 +28313,12 @@
       <c r="O144" t="n">
         <v>3012</v>
       </c>
+      <c r="R144" t="n">
+        <v>4.836223506743738</v>
+      </c>
       <c r="S144" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA144" t="inlineStr">
@@ -28485,9 +28701,12 @@
       <c r="O146" t="n">
         <v>56</v>
       </c>
+      <c r="R146" t="n">
+        <v>0.08991650610147721</v>
+      </c>
       <c r="S146" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA146" t="inlineStr">
@@ -28870,9 +29089,12 @@
       <c r="O148" t="n">
         <v>58</v>
       </c>
+      <c r="R148" t="n">
+        <v>0.09312780989081566</v>
+      </c>
       <c r="S148" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA148" t="inlineStr">
@@ -29255,9 +29477,12 @@
       <c r="O150" t="n">
         <v>1776</v>
       </c>
+      <c r="R150" t="n">
+        <v>2.851637764932562</v>
+      </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA150" t="inlineStr">
@@ -29640,9 +29865,12 @@
       <c r="O152" t="n">
         <v>3191</v>
       </c>
+      <c r="R152" t="n">
+        <v>5.123635195889531</v>
+      </c>
       <c r="S152" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA152" t="inlineStr">
@@ -30025,9 +30253,12 @@
       <c r="O154" t="n">
         <v>37</v>
       </c>
+      <c r="R154" t="n">
+        <v>0.05940912010276172</v>
+      </c>
       <c r="S154" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA154" t="inlineStr">
@@ -30410,9 +30641,12 @@
       <c r="O156" t="n">
         <v>19</v>
       </c>
+      <c r="R156" t="n">
+        <v>0.03050738599871548</v>
+      </c>
       <c r="S156" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA156" t="inlineStr">
@@ -30795,9 +31029,12 @@
       <c r="O158" t="n">
         <v>39</v>
       </c>
+      <c r="R158" t="n">
+        <v>0.06262042389210019</v>
+      </c>
       <c r="S158" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA158" t="inlineStr">
@@ -31180,9 +31417,12 @@
       <c r="O160" t="n">
         <v>775</v>
       </c>
+      <c r="R160" t="n">
+        <v>1.244380218368658</v>
+      </c>
       <c r="S160" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA160" t="inlineStr">
@@ -31565,9 +31805,12 @@
       <c r="O162" t="n">
         <v>338</v>
       </c>
+      <c r="R162" t="n">
+        <v>0.5427103403982017</v>
+      </c>
       <c r="S162" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA162" t="inlineStr">
@@ -31950,9 +32193,12 @@
       <c r="O164" t="n">
         <v>282</v>
       </c>
+      <c r="R164" t="n">
+        <v>0.4527938342967244</v>
+      </c>
       <c r="S164" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA164" t="inlineStr">
@@ -32335,9 +32581,12 @@
       <c r="O166" t="n">
         <v>1199</v>
       </c>
+      <c r="R166" t="n">
+        <v>1.925176621708414</v>
+      </c>
       <c r="S166" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA166" t="inlineStr">
@@ -32720,9 +32969,12 @@
       <c r="O168" t="n">
         <v>154</v>
       </c>
+      <c r="R168" t="n">
+        <v>0.2472703917790623</v>
+      </c>
       <c r="S168" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA168" t="inlineStr">
@@ -33105,9 +33357,12 @@
       <c r="O170" t="n">
         <v>39</v>
       </c>
+      <c r="R170" t="n">
+        <v>0.06262042389210019</v>
+      </c>
       <c r="S170" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA170" t="inlineStr">
@@ -33490,9 +33745,12 @@
       <c r="O172" t="n">
         <v>2079</v>
       </c>
+      <c r="R172" t="n">
+        <v>3.338150289017341</v>
+      </c>
       <c r="S172" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA172" t="inlineStr">
@@ -33875,9 +34133,12 @@
       <c r="O174" t="n">
         <v>29</v>
       </c>
+      <c r="R174" t="n">
+        <v>0.04656390494540783</v>
+      </c>
       <c r="S174" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA174" t="inlineStr">
@@ -34260,9 +34521,12 @@
       <c r="O176" t="n">
         <v>1</v>
       </c>
+      <c r="R176" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S176" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA176" t="inlineStr">
@@ -34645,9 +34909,12 @@
       <c r="O178" t="n">
         <v>365</v>
       </c>
+      <c r="R178" t="n">
+        <v>0.586062941554271</v>
+      </c>
       <c r="S178" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA178" t="inlineStr">
@@ -35030,9 +35297,12 @@
       <c r="O180" t="n">
         <v>2792</v>
       </c>
+      <c r="R180" t="n">
+        <v>4.482980089916507</v>
+      </c>
       <c r="S180" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA180" t="inlineStr">
@@ -35415,9 +35685,12 @@
       <c r="O182" t="n">
         <v>54</v>
       </c>
+      <c r="R182" t="n">
+        <v>0.08670520231213873</v>
+      </c>
       <c r="S182" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA182" t="inlineStr">
@@ -35800,9 +36073,12 @@
       <c r="O184" t="n">
         <v>56</v>
       </c>
+      <c r="R184" t="n">
+        <v>0.08991650610147721</v>
+      </c>
       <c r="S184" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA184" t="inlineStr">
@@ -36185,9 +36461,12 @@
       <c r="O186" t="n">
         <v>9</v>
       </c>
+      <c r="R186" t="n">
+        <v>0.01445086705202312</v>
+      </c>
       <c r="S186" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA186" t="inlineStr">
@@ -36570,9 +36849,12 @@
       <c r="O188" t="n">
         <v>3060</v>
       </c>
+      <c r="R188" t="n">
+        <v>4.913294797687861</v>
+      </c>
       <c r="S188" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA188" t="inlineStr">
@@ -36955,9 +37237,12 @@
       <c r="O190" t="n">
         <v>3030</v>
       </c>
+      <c r="R190" t="n">
+        <v>4.865125240847784</v>
+      </c>
       <c r="S190" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA190" t="inlineStr">
@@ -37340,9 +37625,12 @@
       <c r="O192" t="n">
         <v>44</v>
       </c>
+      <c r="R192" t="n">
+        <v>0.07064868336544637</v>
+      </c>
       <c r="S192" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA192" t="inlineStr">
@@ -37725,9 +38013,12 @@
       <c r="O194" t="n">
         <v>21</v>
       </c>
+      <c r="R194" t="n">
+        <v>0.03371868978805395</v>
+      </c>
       <c r="S194" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA194" t="inlineStr">
@@ -38110,9 +38401,12 @@
       <c r="O196" t="n">
         <v>29</v>
       </c>
+      <c r="R196" t="n">
+        <v>0.04656390494540783</v>
+      </c>
       <c r="S196" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA196" t="inlineStr">
@@ -38495,9 +38789,12 @@
       <c r="O198" t="n">
         <v>666</v>
       </c>
+      <c r="R198" t="n">
+        <v>1.069364161849711</v>
+      </c>
       <c r="S198" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA198" t="inlineStr">
@@ -38880,9 +39177,12 @@
       <c r="O200" t="n">
         <v>369</v>
       </c>
+      <c r="R200" t="n">
+        <v>0.592485549132948</v>
+      </c>
       <c r="S200" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA200" t="inlineStr">
@@ -39265,9 +39565,12 @@
       <c r="O202" t="n">
         <v>632</v>
       </c>
+      <c r="R202" t="n">
+        <v>1.014771997430957</v>
+      </c>
       <c r="S202" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA202" t="inlineStr">
@@ -39650,9 +39953,12 @@
       <c r="O204" t="n">
         <v>1568</v>
       </c>
+      <c r="R204" t="n">
+        <v>2.517662170841362</v>
+      </c>
       <c r="S204" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA204" t="inlineStr">
@@ -40035,9 +40341,12 @@
       <c r="O206" t="n">
         <v>69</v>
       </c>
+      <c r="R206" t="n">
+        <v>0.1107899807321773</v>
+      </c>
       <c r="S206" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA206" t="inlineStr">
@@ -40420,9 +40729,12 @@
       <c r="O208" t="n">
         <v>38</v>
       </c>
+      <c r="R208" t="n">
+        <v>0.06101477199743096</v>
+      </c>
       <c r="S208" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA208" t="inlineStr">
@@ -40805,9 +41117,12 @@
       <c r="O210" t="n">
         <v>3438</v>
       </c>
+      <c r="R210" t="n">
+        <v>5.520231213872832</v>
+      </c>
       <c r="S210" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA210" t="inlineStr">
@@ -41190,9 +41505,12 @@
       <c r="O212" t="n">
         <v>17</v>
       </c>
+      <c r="R212" t="n">
+        <v>0.02729608220937701</v>
+      </c>
       <c r="S212" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA212" t="inlineStr">
@@ -41575,9 +41893,12 @@
       <c r="O214" t="n">
         <v>326</v>
       </c>
+      <c r="R214" t="n">
+        <v>0.5234425176621709</v>
+      </c>
       <c r="S214" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA214" t="inlineStr">
@@ -41960,9 +42281,12 @@
       <c r="O216" t="n">
         <v>2870</v>
       </c>
+      <c r="R216" t="n">
+        <v>4.608220937700707</v>
+      </c>
       <c r="S216" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA216" t="inlineStr">
@@ -42345,9 +42669,12 @@
       <c r="O218" t="n">
         <v>56</v>
       </c>
+      <c r="R218" t="n">
+        <v>0.08991650610147721</v>
+      </c>
       <c r="S218" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA218" t="inlineStr">
@@ -42730,9 +43057,12 @@
       <c r="O220" t="n">
         <v>30</v>
       </c>
+      <c r="R220" t="n">
+        <v>0.04816955684007707</v>
+      </c>
       <c r="S220" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA220" t="inlineStr">
@@ -43115,9 +43445,12 @@
       <c r="O222" t="n">
         <v>138</v>
       </c>
+      <c r="R222" t="n">
+        <v>0.2215799614643545</v>
+      </c>
       <c r="S222" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA222" t="inlineStr">
@@ -43500,9 +43833,12 @@
       <c r="O224" t="n">
         <v>3260</v>
       </c>
+      <c r="R224" t="n">
+        <v>5.234425176621708</v>
+      </c>
       <c r="S224" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA224" t="inlineStr">
@@ -43885,9 +44221,12 @@
       <c r="O226" t="n">
         <v>2975</v>
       </c>
+      <c r="R226" t="n">
+        <v>4.776814386640976</v>
+      </c>
       <c r="S226" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA226" t="inlineStr">
@@ -44270,9 +44609,12 @@
       <c r="O228" t="n">
         <v>48</v>
       </c>
+      <c r="R228" t="n">
+        <v>0.07707129094412331</v>
+      </c>
       <c r="S228" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA228" t="inlineStr">
@@ -44655,9 +44997,12 @@
       <c r="O230" t="n">
         <v>22</v>
       </c>
+      <c r="R230" t="n">
+        <v>0.03532434168272319</v>
+      </c>
       <c r="S230" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA230" t="inlineStr">
@@ -45040,9 +45385,12 @@
       <c r="O232" t="n">
         <v>8</v>
       </c>
+      <c r="R232" t="n">
+        <v>0.01284521515735389</v>
+      </c>
       <c r="S232" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA232" t="inlineStr">
@@ -45425,9 +45773,12 @@
       <c r="O234" t="n">
         <v>641</v>
       </c>
+      <c r="R234" t="n">
+        <v>1.02922286448298</v>
+      </c>
       <c r="S234" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA234" t="inlineStr">
@@ -45810,9 +46161,12 @@
       <c r="O236" t="n">
         <v>292</v>
       </c>
+      <c r="R236" t="n">
+        <v>0.4688503532434168</v>
+      </c>
       <c r="S236" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA236" t="inlineStr">
@@ -46195,9 +46549,12 @@
       <c r="O238" t="n">
         <v>1135</v>
       </c>
+      <c r="R238" t="n">
+        <v>1.822414900449582</v>
+      </c>
       <c r="S238" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA238" t="inlineStr">
@@ -46580,9 +46937,12 @@
       <c r="O240" t="n">
         <v>1017</v>
       </c>
+      <c r="R240" t="n">
+        <v>1.632947976878613</v>
+      </c>
       <c r="S240" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA240" t="inlineStr">
@@ -46965,9 +47325,12 @@
       <c r="O242" t="n">
         <v>25</v>
       </c>
+      <c r="R242" t="n">
+        <v>0.0401412973667309</v>
+      </c>
       <c r="S242" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA242" t="inlineStr">
@@ -47350,9 +47713,12 @@
       <c r="O244" t="n">
         <v>54</v>
       </c>
+      <c r="R244" t="n">
+        <v>0.08670520231213873</v>
+      </c>
       <c r="S244" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA244" t="inlineStr">
@@ -47735,9 +48101,12 @@
       <c r="O246" t="n">
         <v>4125</v>
       </c>
+      <c r="R246" t="n">
+        <v>6.623314065510598</v>
+      </c>
       <c r="S246" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA246" t="inlineStr">
@@ -48120,9 +48489,12 @@
       <c r="O248" t="n">
         <v>5</v>
       </c>
+      <c r="R248" t="n">
+        <v>0.008028259473346179</v>
+      </c>
       <c r="S248" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA248" t="inlineStr">
@@ -48505,9 +48877,12 @@
       <c r="O250" t="n">
         <v>1</v>
       </c>
+      <c r="R250" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA250" t="inlineStr">
@@ -48890,9 +49265,12 @@
       <c r="O252" t="n">
         <v>315</v>
       </c>
+      <c r="R252" t="n">
+        <v>0.5057803468208093</v>
+      </c>
       <c r="S252" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA252" t="inlineStr">
@@ -49275,9 +49653,12 @@
       <c r="O254" t="n">
         <v>2691</v>
       </c>
+      <c r="R254" t="n">
+        <v>4.320809248554913</v>
+      </c>
       <c r="S254" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA254" t="inlineStr">
@@ -49660,9 +50041,12 @@
       <c r="O256" t="n">
         <v>63</v>
       </c>
+      <c r="R256" t="n">
+        <v>0.1011560693641619</v>
+      </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA256" t="inlineStr">
@@ -50045,9 +50429,12 @@
       <c r="O258" t="n">
         <v>34</v>
       </c>
+      <c r="R258" t="n">
+        <v>0.05459216441875402</v>
+      </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA258" t="inlineStr">
@@ -50430,9 +50817,12 @@
       <c r="O260" t="n">
         <v>31</v>
       </c>
+      <c r="R260" t="n">
+        <v>0.04977520873474631</v>
+      </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA260" t="inlineStr">
@@ -50815,9 +51205,12 @@
       <c r="O262" t="n">
         <v>2879</v>
       </c>
+      <c r="R262" t="n">
+        <v>4.62267180475273</v>
+      </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA262" t="inlineStr">
@@ -51200,9 +51593,12 @@
       <c r="O264" t="n">
         <v>3012</v>
       </c>
+      <c r="R264" t="n">
+        <v>4.836223506743738</v>
+      </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA264" t="inlineStr">
@@ -51585,9 +51981,12 @@
       <c r="O266" t="n">
         <v>56</v>
       </c>
+      <c r="R266" t="n">
+        <v>0.08991650610147721</v>
+      </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA266" t="inlineStr">
@@ -51970,9 +52369,12 @@
       <c r="O268" t="n">
         <v>12</v>
       </c>
+      <c r="R268" t="n">
+        <v>0.01926782273603083</v>
+      </c>
       <c r="S268" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA268" t="inlineStr">
@@ -52355,9 +52757,12 @@
       <c r="O270" t="n">
         <v>7</v>
       </c>
+      <c r="R270" t="n">
+        <v>0.01123956326268465</v>
+      </c>
       <c r="S270" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA270" t="inlineStr">
@@ -52740,9 +53145,12 @@
       <c r="O272" t="n">
         <v>1</v>
       </c>
+      <c r="R272" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S272" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA272" t="inlineStr">
@@ -53125,9 +53533,12 @@
       <c r="O274" t="n">
         <v>634</v>
       </c>
+      <c r="R274" t="n">
+        <v>1.017983301220295</v>
+      </c>
       <c r="S274" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA274" t="inlineStr">
@@ -53510,9 +53921,12 @@
       <c r="O276" t="n">
         <v>290</v>
       </c>
+      <c r="R276" t="n">
+        <v>0.4656390494540784</v>
+      </c>
       <c r="S276" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA276" t="inlineStr">
@@ -53895,9 +54309,12 @@
       <c r="O278" t="n">
         <v>1886</v>
       </c>
+      <c r="R278" t="n">
+        <v>3.028259473346179</v>
+      </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA278" t="inlineStr">
@@ -54280,9 +54697,12 @@
       <c r="O280" t="n">
         <v>311</v>
       </c>
+      <c r="R280" t="n">
+        <v>0.4993577392421323</v>
+      </c>
       <c r="S280" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA280" t="inlineStr">
@@ -54665,9 +55085,12 @@
       <c r="O282" t="n">
         <v>15</v>
       </c>
+      <c r="R282" t="n">
+        <v>0.02408477842003853</v>
+      </c>
       <c r="S282" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA282" t="inlineStr">
@@ -55050,9 +55473,12 @@
       <c r="O284" t="n">
         <v>29</v>
       </c>
+      <c r="R284" t="n">
+        <v>0.04656390494540783</v>
+      </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA284" t="inlineStr">
@@ -55435,9 +55861,12 @@
       <c r="O286" t="n">
         <v>3009</v>
       </c>
+      <c r="R286" t="n">
+        <v>4.831406551059731</v>
+      </c>
       <c r="S286" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA286" t="inlineStr">
@@ -55820,9 +56249,12 @@
       <c r="O288" t="n">
         <v>8</v>
       </c>
+      <c r="R288" t="n">
+        <v>0.01284521515735389</v>
+      </c>
       <c r="S288" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA288" t="inlineStr">
@@ -56205,9 +56637,12 @@
       <c r="O290" t="n">
         <v>256</v>
       </c>
+      <c r="R290" t="n">
+        <v>0.4110468850353243</v>
+      </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA290" t="inlineStr">
@@ -56590,9 +57025,12 @@
       <c r="O292" t="n">
         <v>2179</v>
       </c>
+      <c r="R292" t="n">
+        <v>3.498715478484264</v>
+      </c>
       <c r="S292" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA292" t="inlineStr">
@@ -56975,9 +57413,12 @@
       <c r="O294" t="n">
         <v>54</v>
       </c>
+      <c r="R294" t="n">
+        <v>0.08670520231213873</v>
+      </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA294" t="inlineStr">
@@ -57360,9 +57801,12 @@
       <c r="O296" t="n">
         <v>20</v>
       </c>
+      <c r="R296" t="n">
+        <v>0.03211303789338472</v>
+      </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA296" t="inlineStr">
@@ -57745,9 +58189,12 @@
       <c r="O298" t="n">
         <v>2</v>
       </c>
+      <c r="R298" t="n">
+        <v>0.003211303789338471</v>
+      </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA298" t="inlineStr">
@@ -58130,9 +58577,12 @@
       <c r="O300" t="n">
         <v>2491</v>
       </c>
+      <c r="R300" t="n">
+        <v>3.999678869621067</v>
+      </c>
       <c r="S300" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA300" t="inlineStr">
@@ -58515,9 +58965,12 @@
       <c r="O302" t="n">
         <v>2947</v>
       </c>
+      <c r="R302" t="n">
+        <v>4.731856133590238</v>
+      </c>
       <c r="S302" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA302" t="inlineStr">
@@ -58900,9 +59353,12 @@
       <c r="O304" t="n">
         <v>43</v>
       </c>
+      <c r="R304" t="n">
+        <v>0.06904303147077713</v>
+      </c>
       <c r="S304" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA304" t="inlineStr">
@@ -59285,9 +59741,12 @@
       <c r="O306" t="n">
         <v>1</v>
       </c>
+      <c r="R306" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S306" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA306" t="inlineStr">
@@ -59670,9 +60129,12 @@
       <c r="O308" t="n">
         <v>10</v>
       </c>
+      <c r="R308" t="n">
+        <v>0.01605651894669236</v>
+      </c>
       <c r="S308" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA308" t="inlineStr">
@@ -60055,9 +60517,12 @@
       <c r="O310" t="n">
         <v>612</v>
       </c>
+      <c r="R310" t="n">
+        <v>0.9826589595375723</v>
+      </c>
       <c r="S310" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA310" t="inlineStr">
@@ -60440,9 +60905,12 @@
       <c r="O312" t="n">
         <v>232</v>
       </c>
+      <c r="R312" t="n">
+        <v>0.3725112395632627</v>
+      </c>
       <c r="S312" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA312" t="inlineStr">
@@ -60825,9 +61293,12 @@
       <c r="O314" t="n">
         <v>2066</v>
       </c>
+      <c r="R314" t="n">
+        <v>3.317276814386641</v>
+      </c>
       <c r="S314" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA314" t="inlineStr">
@@ -61210,9 +61681,12 @@
       <c r="O316" t="n">
         <v>206</v>
       </c>
+      <c r="R316" t="n">
+        <v>0.3307642903018626</v>
+      </c>
       <c r="S316" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA316" t="inlineStr">
@@ -61595,9 +62069,12 @@
       <c r="O318" t="n">
         <v>13</v>
       </c>
+      <c r="R318" t="n">
+        <v>0.02087347463070006</v>
+      </c>
       <c r="S318" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA318" t="inlineStr">
@@ -61980,9 +62457,12 @@
       <c r="O320" t="n">
         <v>42</v>
       </c>
+      <c r="R320" t="n">
+        <v>0.0674373795761079</v>
+      </c>
       <c r="S320" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA320" t="inlineStr">
@@ -62365,9 +62845,12 @@
       <c r="O322" t="n">
         <v>2135</v>
       </c>
+      <c r="R322" t="n">
+        <v>3.428066795118818</v>
+      </c>
       <c r="S322" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA322" t="inlineStr">
@@ -62750,9 +63233,12 @@
       <c r="O324" t="n">
         <v>13</v>
       </c>
+      <c r="R324" t="n">
+        <v>0.02087347463070006</v>
+      </c>
       <c r="S324" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA324" t="inlineStr">
@@ -63135,9 +63621,12 @@
       <c r="O326" t="n">
         <v>0</v>
       </c>
+      <c r="R326" t="n">
+        <v>0</v>
+      </c>
       <c r="S326" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA326" t="inlineStr">
@@ -63520,9 +64009,12 @@
       <c r="O328" t="n">
         <v>212</v>
       </c>
+      <c r="R328" t="n">
+        <v>0.3403982016698779</v>
+      </c>
       <c r="S328" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA328" t="inlineStr">
@@ -63905,9 +64397,12 @@
       <c r="O330" t="n">
         <v>2615</v>
       </c>
+      <c r="R330" t="n">
+        <v>4.198779704560051</v>
+      </c>
       <c r="S330" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA330" t="inlineStr">
@@ -64290,9 +64785,12 @@
       <c r="O332" t="n">
         <v>37</v>
       </c>
+      <c r="R332" t="n">
+        <v>0.05940912010276172</v>
+      </c>
       <c r="S332" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA332" t="inlineStr">
@@ -64675,9 +65173,12 @@
       <c r="O334" t="n">
         <v>16</v>
       </c>
+      <c r="R334" t="n">
+        <v>0.02569043031470777</v>
+      </c>
       <c r="S334" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA334" t="inlineStr">
@@ -65060,9 +65561,12 @@
       <c r="O336" t="n">
         <v>1631</v>
       </c>
+      <c r="R336" t="n">
+        <v>2.618818240205524</v>
+      </c>
       <c r="S336" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA336" t="inlineStr">
@@ -65445,9 +65949,12 @@
       <c r="O338" t="n">
         <v>2943</v>
       </c>
+      <c r="R338" t="n">
+        <v>4.72543352601156</v>
+      </c>
       <c r="S338" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA338" t="inlineStr">
@@ -65830,9 +66337,12 @@
       <c r="O340" t="n">
         <v>56</v>
       </c>
+      <c r="R340" t="n">
+        <v>0.08991650610147721</v>
+      </c>
       <c r="S340" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA340" t="inlineStr">
@@ -66215,9 +66725,12 @@
       <c r="O342" t="n">
         <v>2</v>
       </c>
+      <c r="R342" t="n">
+        <v>0.003211303789338471</v>
+      </c>
       <c r="S342" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA342" t="inlineStr">
@@ -66600,9 +67113,12 @@
       <c r="O344" t="n">
         <v>10</v>
       </c>
+      <c r="R344" t="n">
+        <v>0.01605651894669236</v>
+      </c>
       <c r="S344" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA344" t="inlineStr">
@@ -66985,9 +67501,12 @@
       <c r="O346" t="n">
         <v>635</v>
       </c>
+      <c r="R346" t="n">
+        <v>1.019588953114965</v>
+      </c>
       <c r="S346" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA346" t="inlineStr">
@@ -67370,9 +67889,12 @@
       <c r="O348" t="n">
         <v>250</v>
       </c>
+      <c r="R348" t="n">
+        <v>0.4014129736673089</v>
+      </c>
       <c r="S348" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA348" t="inlineStr">
@@ -67755,9 +68277,12 @@
       <c r="O350" t="n">
         <v>2313</v>
       </c>
+      <c r="R350" t="n">
+        <v>3.713872832369942</v>
+      </c>
       <c r="S350" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA350" t="inlineStr">
@@ -68140,9 +68665,12 @@
       <c r="O352" t="n">
         <v>407</v>
       </c>
+      <c r="R352" t="n">
+        <v>0.6535003211303789</v>
+      </c>
       <c r="S352" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA352" t="inlineStr">
@@ -68525,9 +69053,12 @@
       <c r="O354" t="n">
         <v>14</v>
       </c>
+      <c r="R354" t="n">
+        <v>0.0224791265253693</v>
+      </c>
       <c r="S354" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA354" t="inlineStr">
@@ -68910,9 +69441,12 @@
       <c r="O356" t="n">
         <v>18</v>
       </c>
+      <c r="R356" t="n">
+        <v>0.02890173410404624</v>
+      </c>
       <c r="S356" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA356" t="inlineStr">
@@ -69295,9 +69829,12 @@
       <c r="O358" t="n">
         <v>2195</v>
       </c>
+      <c r="R358" t="n">
+        <v>3.524405908798973</v>
+      </c>
       <c r="S358" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA358" t="inlineStr">
@@ -69680,9 +70217,12 @@
       <c r="O360" t="n">
         <v>49</v>
       </c>
+      <c r="R360" t="n">
+        <v>0.07867694283879255</v>
+      </c>
       <c r="S360" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA360" t="inlineStr">
@@ -70065,9 +70605,12 @@
       <c r="O362" t="n">
         <v>1</v>
       </c>
+      <c r="R362" t="n">
+        <v>0.001605651894669236</v>
+      </c>
       <c r="S362" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA362" t="inlineStr">
@@ -70450,9 +70993,12 @@
       <c r="O364" t="n">
         <v>196</v>
       </c>
+      <c r="R364" t="n">
+        <v>0.3147077713551702</v>
+      </c>
       <c r="S364" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA364" t="inlineStr">
@@ -70835,9 +71381,12 @@
       <c r="O366" t="n">
         <v>2385</v>
       </c>
+      <c r="R366" t="n">
+        <v>3.829479768786127</v>
+      </c>
       <c r="S366" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA366" t="inlineStr">
@@ -71220,9 +71769,12 @@
       <c r="O368" t="n">
         <v>54</v>
       </c>
+      <c r="R368" t="n">
+        <v>0.08670520231213873</v>
+      </c>
       <c r="S368" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA368" t="inlineStr">
@@ -71605,9 +72157,12 @@
       <c r="O370" t="n">
         <v>43</v>
       </c>
+      <c r="R370" t="n">
+        <v>0.06904303147077713</v>
+      </c>
       <c r="S370" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA370" t="inlineStr">
@@ -71990,9 +72545,12 @@
       <c r="O372" t="n">
         <v>874</v>
       </c>
+      <c r="R372" t="n">
+        <v>1.403339755940912</v>
+      </c>
       <c r="S372" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA372" t="inlineStr">
@@ -72375,9 +72933,12 @@
       <c r="O374" t="n">
         <v>2301</v>
       </c>
+      <c r="R374" t="n">
+        <v>3.694605009633911</v>
+      </c>
       <c r="S374" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA374" t="inlineStr">
@@ -72760,9 +73321,12 @@
       <c r="O376" t="n">
         <v>15</v>
       </c>
+      <c r="R376" t="n">
+        <v>0.02408477842003853</v>
+      </c>
       <c r="S376" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA376" t="inlineStr">
@@ -73145,9 +73709,12 @@
       <c r="O378" t="n">
         <v>5</v>
       </c>
+      <c r="R378" t="n">
+        <v>0.008028259473346179</v>
+      </c>
       <c r="S378" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA378" t="inlineStr">
@@ -73530,9 +74097,12 @@
       <c r="O380" t="n">
         <v>26</v>
       </c>
+      <c r="R380" t="n">
+        <v>0.04174694926140013</v>
+      </c>
       <c r="S380" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA380" t="inlineStr">
@@ -73915,9 +74485,12 @@
       <c r="O382" t="n">
         <v>609</v>
       </c>
+      <c r="R382" t="n">
+        <v>0.9778420038535646</v>
+      </c>
       <c r="S382" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA382" t="inlineStr">
@@ -74300,9 +74873,12 @@
       <c r="O384" t="n">
         <v>215</v>
       </c>
+      <c r="R384" t="n">
+        <v>0.3452151573538857</v>
+      </c>
       <c r="S384" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA384" t="inlineStr">
@@ -74685,9 +75261,12 @@
       <c r="O386" t="n">
         <v>302</v>
       </c>
+      <c r="R386" t="n">
+        <v>0.4849068721901091</v>
+      </c>
       <c r="S386" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA386" t="inlineStr">
@@ -75070,9 +75649,12 @@
       <c r="O388" t="n">
         <v>615</v>
       </c>
+      <c r="R388" t="n">
+        <v>0.9874759152215801</v>
+      </c>
       <c r="S388" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA388" t="inlineStr">
@@ -75455,9 +76037,12 @@
       <c r="O390" t="n">
         <v>12</v>
       </c>
+      <c r="R390" t="n">
+        <v>0.01926782273603083</v>
+      </c>
       <c r="S390" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA390" t="inlineStr">
@@ -75840,9 +76425,12 @@
       <c r="O392" t="n">
         <v>24</v>
       </c>
+      <c r="R392" t="n">
+        <v>0.03853564547206165</v>
+      </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA392" t="inlineStr">
@@ -76225,9 +76813,12 @@
       <c r="O394" t="n">
         <v>1366</v>
       </c>
+      <c r="R394" t="n">
+        <v>2.193320488118176</v>
+      </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA394" t="inlineStr">
@@ -76610,9 +77201,12 @@
       <c r="O396" t="n">
         <v>28</v>
       </c>
+      <c r="R396" t="n">
+        <v>0.0449582530507386</v>
+      </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA396" t="inlineStr">
@@ -76995,9 +77589,12 @@
       <c r="O398" t="n">
         <v>0</v>
       </c>
+      <c r="R398" t="n">
+        <v>0</v>
+      </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA398" t="inlineStr">
@@ -77380,9 +77977,12 @@
       <c r="O400" t="n">
         <v>156</v>
       </c>
+      <c r="R400" t="n">
+        <v>0.2504816955684008</v>
+      </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA400" t="inlineStr">
@@ -77765,9 +78365,12 @@
       <c r="O402" t="n">
         <v>1609</v>
       </c>
+      <c r="R402" t="n">
+        <v>2.5834938985228</v>
+      </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA402" t="inlineStr">
@@ -78150,9 +78753,12 @@
       <c r="O404" t="n">
         <v>43</v>
       </c>
+      <c r="R404" t="n">
+        <v>0.06904303147077713</v>
+      </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA404" t="inlineStr">
@@ -78535,9 +79141,12 @@
       <c r="O406" t="n">
         <v>31</v>
       </c>
+      <c r="R406" t="n">
+        <v>0.04977520873474631</v>
+      </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA406" t="inlineStr">
@@ -78920,9 +79529,12 @@
       <c r="O408" t="n">
         <v>461</v>
       </c>
+      <c r="R408" t="n">
+        <v>0.7402055234425177</v>
+      </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA408" t="inlineStr">
@@ -79305,9 +79917,12 @@
       <c r="O410" t="n">
         <v>1356</v>
       </c>
+      <c r="R410" t="n">
+        <v>2.177263969171483</v>
+      </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA410" t="inlineStr">
@@ -79690,9 +80305,12 @@
       <c r="O412" t="n">
         <v>11</v>
       </c>
+      <c r="R412" t="n">
+        <v>0.01766217084136159</v>
+      </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA412" t="inlineStr">
@@ -80075,9 +80693,12 @@
       <c r="O414" t="n">
         <v>32</v>
       </c>
+      <c r="R414" t="n">
+        <v>0.05138086062941554</v>
+      </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA414" t="inlineStr">
@@ -80460,9 +81081,12 @@
       <c r="O416" t="n">
         <v>505</v>
       </c>
+      <c r="R416" t="n">
+        <v>0.8108542068079639</v>
+      </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA416" t="inlineStr">
@@ -80845,9 +81469,12 @@
       <c r="O418" t="n">
         <v>149</v>
       </c>
+      <c r="R418" t="n">
+        <v>0.2392421323057161</v>
+      </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA418" t="inlineStr">
@@ -81230,9 +81857,12 @@
       <c r="O420" t="n">
         <v>37</v>
       </c>
+      <c r="R420" t="n">
+        <v>0.05940912010276172</v>
+      </c>
       <c r="S420" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA420" t="inlineStr">
@@ -81615,9 +82245,12 @@
       <c r="O422" t="n">
         <v>815</v>
       </c>
+      <c r="R422" t="n">
+        <v>1.308606294155427</v>
+      </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA422" t="inlineStr">
@@ -82000,9 +82633,12 @@
       <c r="O424" t="n">
         <v>8</v>
       </c>
+      <c r="R424" t="n">
+        <v>0.01284521515735389</v>
+      </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA424" t="inlineStr">
@@ -82385,9 +83021,12 @@
       <c r="O426" t="n">
         <v>22</v>
       </c>
+      <c r="R426" t="n">
+        <v>0.03532434168272319</v>
+      </c>
       <c r="S426" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA426" t="inlineStr">
@@ -82770,9 +83409,12 @@
       <c r="O428" t="n">
         <v>776</v>
       </c>
+      <c r="R428" t="n">
+        <v>1.245985870263327</v>
+      </c>
       <c r="S428" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA428" t="inlineStr">
@@ -83155,9 +83797,12 @@
       <c r="O430" t="n">
         <v>14</v>
       </c>
+      <c r="R430" t="n">
+        <v>0.0224791265253693</v>
+      </c>
       <c r="S430" t="inlineStr">
         <is>
-          <t>missing_population</t>
+          <t>nbs_computed</t>
         </is>
       </c>
       <c r="AA430" t="inlineStr">

</xml_diff>